<commit_message>
nowy parser, podzial opisu na czesci, data rozpoznanie, dane kliniczne , opis i wniosi
</commit_message>
<xml_diff>
--- a/pacjenci/ADAM HAZIK.xlsx
+++ b/pacjenci/ADAM HAZIK.xlsx
@@ -413,38 +413,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Nr badania</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Data badania</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Nr badania</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Etap leczenia</t>
+          <t>Problem kliniczny</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Linia leczenia</t>
+          <t>Zakres badania</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Rozpoznanie</t>
+          <t>Opis badania</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Opis</t>
+          <t>Wnioski</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -452,328 +452,236 @@
           <t>SUVmax</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Ocena odpowiedzi</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Deauville</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Wnioski</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>13.03.2023</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena stopnia zaawansowania.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud Akwizycję przeprowadzono  po  59min od podania 18F-FDG. Glikemia: 94mg%</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Fizjologiczny metabolizm FDG w obrębie głowy i szyi. Dyskretne pogrubienie błony śluzowej w prawej zatoce szczękowej.  Klatka piersiowa i śródpiersie: Duży aktywny metabolicznie naciek w śródpiersiu przednim po stronie lewej z niewykluczonym naciekiem przyległego miąższu płuc wielkości wg PET 71x76mm, SUV max 19,9.  Aktywne metabolicznie węzły chłonne: - w śródpiersiu przednim po stronie prawej średnicy wg PET do 21mm, SUV max do 6,0, - okna aortalno-płucnego oraz przytchawicze górne lewe wielkości wg PET do  37x17mm, SUV max do 11,8, - wnęki płuca lewego średnicy wg PET do 24mm, SUV max do 11,7, - w zachyłku przeponowo-żebrowym po stronie lewej średnicy wg PET 21mm, SUV max 8,6. Aktywny metabolicznie obszar w ścianie klatki piersiowej po stronie lewej przechodzący przez mięsień piersiowy większy, SUV max do 4,6 - w pierwszej kolejności kanał biopsyjny. Poza tym fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Płyn w lewej jamie opłucnowej grubości płaszcza do 21mm.   Brzuch i miednica: Rozlana aktywność metaboliczna w topografii żołądka, SUV max do 5,7 - w pierwszej kolejności czynnościowa.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy.  Układ kostny: Rozlanie niejednorodny metabolizm FDG w układzie kostnym - w pierwszej kolejności związany ze stosowanym leczeniem.  Wartości referencyjne: MBPS SUVmax 1,4,  Prawy płat wątroby SUVmax do 4,9.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG uwidoczniono aktywną metabolicznie chorobę chłoniakową w zlokalizowaną w śródpiersiu przednim po stronie lewej z niewykluczonym objęciem płuca lewego oraz węzłów chłonnych po jednej stronie przepony.</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>19.9</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Nie dotyczy</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Aktywna metabolicznie choroba przed rozpoczęciem leczenia. Badanie wyjściowe stanowiące punkt odniesienia.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>06.06.2023</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Wczesna ocena odpowiedzi po 2 cyklach SBVD. Badanie kliniczne RAFTING.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 59min od podania 18F-FDG. Glikemia: 89mg%.</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych. Drobne zgrubienia błony śluzowej w zachyłku zębodołowym prawej zatoki szczękowej.  Klatka piersiowa i śródpiersie: Pobudzenie metaboliczne w topografii struktur ściany klatki piersiowej, lewobocznie od linii pośrodkowej, przechodzący przez mięsień piersiowy większy, SUV max do 4,5 - w pierwszej kolejności kanał biopsyjny. Masy miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo, wielkości ok. 69x35x62mm [SUV max do 3,1]-do kontroli. Poza tym fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Pasmowate zmiany miąższowo-włókniste przyśródpiersiowo w płacie górnym płuca lewego-resztkowe zmiany naciekowe.  Brzuch i miednica: Rozlanie wzmożona aktywność metaboliczna w topografii żołądka, SUV max do 7,6 - w pierwszej kolejności czynnościowa.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne obustronnie, wielkości do 9x6mm. Dość liczne drobne węzły chłonne pachwinowe obustronnie.  Układ kostny: Fizjologiczny metabolizm FDG w układzie kostnym. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 5mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Wartości referencyjne: MBPS SUVmax 2,2;  Prawy płat wątroby SUVmax do 3,2.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG uwidoczniono bardzo dobrą odpowiedź metaboliczną choroby chłoniakowej na stosowane leczenie.  Masy miękkotkankowe w śródpiersiu - do kontroli. Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G3" t="n">
         <v>7.6</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>23.08.2023</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena skutków leczenia.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 57min od podania 18F-FDG. Glikemia: 89mg%.</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych.  Klatka piersiowa i śródpiersie: Fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Częściowo rozfragmentowane masy miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo, wielkości do ok. 52x31x37mm [Im. TK 280] - do kontroli. Pasmowate zmiany miąższowo-włókniste przyśródpiersiowo w płacie górnym płuca lewego-nadal utrzymujące się reszkowe zmiany naciekowe - do kontroli w badaniu TK KLP z kontrastem dożylnym. Obwodowe zmiany włókniste w płacie górnym płuca lewego. Niewielkie zmiany miąższowo-włókniste nadprzeponowo w segm. 10 płuca prawego. Niewielkie zmiany włókniste obustronnie nadprzeponowo.  Brzuch i miednica: Rozlanie wzmożona aktywność metaboliczna w topografii żołądka, SUV max do 6,1 - w pierwszej kolejności czynnościowa.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne i pachwinowe obustronnie.  Układ kostny: Fizjologiczny metabolizm FDG w układzie kostnym. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 5mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Wartości referencyjne: MBPS SUVmax 2,0; Prawy płat wątroby SUVmax do 3,2.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG uwidoczniono bardzo dobrą odpowiedź metaboliczną choroby chłoniakowej na stosowane leczenie.  Masy miękkotkankowe w śródpiersiu i zmiany naciekowe w płacie górnym płuca lewego - do kontroli. Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G4" t="n">
         <v>6.1</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>05.03.2024</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>4</v>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena remisji choroby.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 57min od podania 18F-FDG. Glikemia: 74mg%.</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych.  Klatka piersiowa i śródpiersie: Aktywny metabolicznie obszar miękkotkankowy przy pniu płucnym, po stronie lewej, wielkości 11mm wg PET, SUV max 4,4 - węzeł chłonny? ogniskowa aktywność w większej masie miękkotkankowej?.  Poza tym fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Częściowo rozfragmentowane masy miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo, wielkości do ok. 22x19mm [Im. TK 294] - do kontroli. Obwodowe zmiany włókniste w płacie górnym płuca lewego. Niewielkie zmiany miąższowo-włókniste nadprzeponowo w segm. 10 płuca prawego. Niewielkie zmiany włókniste obustronnie nadprzeponowo.  Brzuch i miednica: Rozlanie wzmożona aktywność metaboliczna w topografii żołądka - w pierwszej kolejności czynnościowa.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne i pachwinowe obustronnie.  Układ kostny: Pobudzenie metaboliczne w topografii gojącego się złamania lewego wyrostka poprzecznego kręgu L3, SUV max 3,5- do kontroli.  Poza tym fizjologiczny metabolizm FDG w układzie kostnym. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 6mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Wartości referencyjne: MBPS SUVmax do 1,4; Prawy płat wątroby SUVmax do 2,6.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG uwidoczniono aktywny metabolicznie obszar miękkotkankowy przy pniu płucnym, po stronie lewej - węzeł chłonny? ogniskowa aktywność w większej masie miękkotkankowej? - podejrzenie wznowy choroby. Pobudzenie metaboliczne w topografii gojącego się złamania lewego wyrostka poprzecznego kręgu L3 - do kontroli.  Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G5" t="n">
         <v>4.4</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>12.08.2024</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>5</v>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena remisji choroby.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 57min od podania 18F-FDG. Glikemia: 97mg%.</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych.  Klatka piersiowa i śródpiersie: Fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Częściowo rozfragmentowane masy miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo, wielkości do ok. 19x16mm [Im. TK 289] - do kontroli. Obwodowe zmiany włókniste w płacie górnym płuca lewego. Nieregularny guzek w części podstawnej segm. 3 prawego płuca, przy szczelinie międzypłatowej, wielkości 11x6mm. Obwodowo os niego - drobniejszy, ok. 5x3mm. Niewielkie zmiany miąższowe w segm. 4/5 płuca lewego. Drobne zmiany miąższowo-włókniste nadprzeponowo w segm. 10 płuca prawego. Niewielkie zmiany włókniste obustronnie nadprzeponowo.  Brzuch i miednica: Rozlanie wzmożona aktywność metaboliczna w topografii żołądka - w pierwszej kolejności czynnościowa.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne i pachwinowe obustronnie.  Układ kostny: Fizjologiczny metabolizm FDG w układzie kostnym. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Nieregularne obrysy lewego wyrostka poprzecznego kręgu Th10 oraz przykręgosłupowego odcinka lewego żebra X - stan po urazie? Niewielka dyskopatia na poziomie L5/S1. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 6mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Wartości referencyjne: MBPS SUVmax do 1,7; Prawy płat wątroby SUVmax do 2,4.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG nie uwidoczniono cech aktywnej metabolicznie choroby chłoniakowej.   Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>2.4</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>23.01.2025</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>6</v>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena na zakończenie leczenia w ramach badania RAFTING.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 59min od podania 18F-FDG. Glikemia: 90mg%.</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Pobudzenie metaboliczne w topografii pojedynczych, drobnych węzłów chłonnych przedziału 2 obustronnie wielkości do 9x6mm, SUV max do 2,4. Poza tym fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych. Drobne polipowate zgrubienie błony śluzowej w zachyłku zębodołowym prawej zatoki szczękowej. Bardzo drobne przyścienne zgrubienie błony śluzowej w lewej zatoce szczękowej.  Klatka piersiowa i śródpiersie: Fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Drobne obszary miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo oraz pojedynczy, wydatniejszy lewobocznie od linii pośrodkowej, wielkości do ok. 14x16mm - do kontroli. Obwodowe zmiany włókniste w płacie górnym płuca lewego. Nieregularny, aktualnie słabo wysycony guzek w części podstawnej segm. 3 prawego płuca, przy szczelinie międzypłatowej, wielkości 10x5mm. Obwodowo od niego - drobniejszy, ok. 4x3mm. Drobne zmiany włókniste w segm. 4/5 płuca lewego. Niewielkie zmiany włókniste obustronnie nadprzeponowo.  Brzuch i miednica: Niejednorodne pobudzenie metaboliczne w topografii żołądka - w pierwszej kolejności czynnościowo.  Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne i  pachwinowe wielkości do 10x8mm.  Układ kostny: Fizjologiczny metabolizm FDG w układzie kostnym. Zniesienie fizjologicznej lordozy, cechy niestabilności oraz łukowato kyfotyczne ustawienie kręgosłupa szyjnego. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Nieregularne obrysy lewego wyrostka poprzecznego kręgu Th10 oraz przykręgosłupowego odcinka lewego żebra X - stan po urazie? Niewielka dyskopatia na poziomie L5/S1. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 6mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Inne: Rozlanie zwiększona aktywność metaboliczna w mięśniach- do oceny z całością obrazu klinicznego.   Wartości referencyjne: MBPS SUVmax do 1,0; Prawy płat wątroby SUVmax do 1,4.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG nie uwidoczniono jednoznacznych cech aktywnej metabolicznie choroby chłoniakowej. Pobudzenie metaboliczne w topografii pojedynczych, drobnych węzłów chłonnych przedziału 2 szyi obustronnie - wymaga kontroli. Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>2.4</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>08.04.2025</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>7</v>
-      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>Chłoniak Hodgkina. Ocena remisji choroby.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>od szczytu głowy do 1/3 ud. Akwizycję przeprowadzono  po 59 min od podania 18F-FDG. Glikemia: 96mg%.</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>HL</t>
+          <t>: Symetrycznie wzmożona aktywność metaboliczna w topografii struktur pierścienia Waldeyera, SUV max 9,0. Pobudzenie metaboliczne w topografii pojedynczych węzłów chłonnych przedziału 2 obustronnie, wielkości do 9x6mm, SUV max do 3,1 - w pierwszej kolejności odczynowe. Poza tym fizjologiczny metabolizm FDG w obrębie głowy i szyi. Hypoplazja zatok czołowych. Drobne polipowate zgrubienie błony śluzowej w zachyłku zębodołowym prawej zatoki szczękowej. Drobne przyścienne zgrubienia błony śluzowej w lewej zatoce szczękowej.  Klatka piersiowa i śródpiersie: Fizjologiczny metabolizm FDG w narządach klatki piersiowej i śródpiersia. Drobne obszary miękkotkankowe w śródpiersiu przednim po stronie lewej i nieco pośrodkowo oraz pojedynczy, wydatniejszy lewobocznie od linii pośrodkowej, wielkości do ok. 15x17mm. Obwodowe i przyśródpiersiowe zmiany włókniste w płacie górnym płuca lewego. Nieregularny,  słabo wysycony guzek w części podstawnej segm. 3 prawego płuca, przy szczelinie międzypłatowej, wielkości 9x5mm. Obwodowo od niego - drobniejszy, ok. 4x3mm. Drobne zmiany włókniste w segm. 4/5 płuca lewego. Niewielkie zmiany włókniste obustronnie nadprzeponowo.  Brzuch i miednica: Niejednorodne pobudzenie metaboliczne w topografii żołądka, SUV max do 6,0 - w pierwszej kolejności czynnościowe/odczynowe.  Odcinkowo wzmożona aktywność metaboliczna w topografii pętli jelitowych, zwłaszcza położonych w miednicy, SUV max do 7,5 - czynnościowa?   Poza tym fizjologiczny metabolizm FDG w narządach jamy brzusznej i miednicy. Drobne węzły chłonne przyaortalne i  pachwinowe obustronnie, wielkości do 9x7mm.  Układ kostny: Fizjologiczny metabolizm FDG w układzie kostnym. Zniesienie fizjologicznej lordozy, cechy niestabilności oraz łukowato kyfotyczne ustawienie kręgosłupa szyjnego. Spłycenie fizjologicznych krzywizn kręgosłupa. Os sacrum arcuatum. Nieregularne obrysy lewego wyrostka poprzecznego kręgu Th10 oraz przykręgosłupowego odcinka lewego żebra X - stan po urazie? Drobna retrolisteza i niewielka dyskopatia na poziomie L5/S1. Drobne zmiany wytwórcze w stawach krzyżowo-biodrowych. Ok. 6mm miernie sklerotyczny obszar i drobna wyspa kostna w trzonie prawej kości biodrowej.  Wartości referencyjne: MBPS SUVmax do 1,3; Prawy płat wątroby SUVmax do 2,5.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Do oceny</t>
+          <t>Badaniem PET/CT z 18F-FDG nie uwidoczniono jednoznacznych cech obecności aktywnej metabolicznie choroby chłoniakowej.  Poza tym jak w opisie powyżej.</t>
         </is>
       </c>
       <c r="G8" t="n">
         <v>9</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>4 - utrzymujący się wychwyt patologiczny</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Stabilizacja choroby. Klasyfikacja Lugano: Stable Disease (SD) - stabilizacja choroby. Deauville: 4 - utrzymujący się wychwyt patologiczny.</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>